<commit_message>
Update October actuals and tech count in Goals sheet
October actual revenue now $2,530; technician count updated to 4
after Rylan and Jayce were let go.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D87LwuWDcN4nTXwvgo4Xse
</commit_message>
<xml_diff>
--- a/Coastline_Goals_Sep_Dec_2026.xlsx
+++ b/Coastline_Goals_Sep_Dec_2026.xlsx
@@ -685,7 +685,9 @@
       <c r="C7" s="6" t="n">
         <v>12000</v>
       </c>
-      <c r="D7" s="10" t="inlineStr"/>
+      <c r="D7" s="7" t="n">
+        <v>2530</v>
+      </c>
       <c r="E7" s="8">
         <f>IF(D7="","",D7/B7)</f>
         <v/>
@@ -1227,7 +1229,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Drop Meta ads plan, switch to PPC + LSA for winter
Scratched the Oct 14 Meta ceramic coating ad launch. LSA is
performing well as-is; PPC now launches in December instead.
Updated marketing goals, key dates, and October ad budget note.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D87LwuWDcN4nTXwvgo4Xse
</commit_message>
<xml_diff>
--- a/Coastline_Goals_Sep_Dec_2026.xlsx
+++ b/Coastline_Goals_Sep_Dec_2026.xlsx
@@ -718,7 +718,7 @@
       </c>
       <c r="P7" s="5" t="inlineStr">
         <is>
-          <t>~$450 Meta (from Oct 14)</t>
+          <t>Google LSA only (Meta dropped)</t>
         </is>
       </c>
     </row>
@@ -812,7 +812,7 @@
       </c>
       <c r="P9" s="5" t="inlineStr">
         <is>
-          <t>~$2,000</t>
+          <t>~$2,000 (PPC launches + LSA)</t>
         </is>
       </c>
     </row>
@@ -1057,18 +1057,18 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Meta ceramic coating ads</t>
+          <t>PPC + LSA ads (winter push)</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>Live Oct 14</t>
+          <t>PPC live Dec, LSA ongoing</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>Lead Form ads, 1 new creative a week.</t>
+          <t>LSA performing well as-is; PPC launches December instead of Meta.</t>
         </is>
       </c>
     </row>
@@ -1372,7 +1372,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Meta ceramic coating ads live.</t>
+          <t>(Scratched — Meta ads plan dropped. Keep closing leads from LSA for the rest of October.)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>

</xml_diff>

<commit_message>
Log October revenue at $6,456 in Goals sheet, update Drive links
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XeYkWCpV7g2ezgB3AXjkpD
</commit_message>
<xml_diff>
--- a/Coastline_Goals_Sep_Dec_2026.xlsx
+++ b/Coastline_Goals_Sep_Dec_2026.xlsx
@@ -647,9 +647,7 @@
         <f>IF(D6="","",D6/B6)</f>
         <v/>
       </c>
-      <c r="F6" t="inlineStr"/>
       <c r="G6" s="9" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
       <c r="I6" s="9" t="inlineStr"/>
       <c r="J6" s="8">
         <f>IF(OR(I6="",I6=0,G6=""),"",G6/I6)</f>
@@ -686,7 +684,7 @@
         <v>12000</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>2530</v>
+        <v>6456</v>
       </c>
       <c r="E7" s="8">
         <f>IF(D7="","",D7/B7)</f>
@@ -975,7 +973,6 @@
           <t>100%</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Reply within 24 hours, good or bad.</t>
@@ -993,7 +990,6 @@
           <t>1 a week (14 posts)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
       <c r="D8" s="5" t="inlineStr">
         <is>
           <t>Post the current offer + before-and-afters.</t>
@@ -1011,7 +1007,6 @@
           <t>1 a day (about 95)</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>One before-and-after or hook video a day.</t>
@@ -1029,7 +1024,6 @@
           <t>Under 5 minutes</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
       <c r="D10" s="5" t="inlineStr">
         <is>
           <t>GoHighLevel instant text 24/7 + call.</t>
@@ -1047,7 +1041,6 @@
           <t>40%+</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
       <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Close On The Spot sheet. Track every quote.</t>
@@ -1065,7 +1058,6 @@
           <t>PPC live Dec, LSA ongoing</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
       <c r="D12" s="5" t="inlineStr">
         <is>
           <t>LSA performing well as-is; PPC launches December instead of Meta.</t>
@@ -1083,7 +1075,6 @@
           <t>Live Nov 1</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
       <c r="D13" s="5" t="inlineStr">
         <is>
           <t>$15–25/day, landing page in GoHighLevel.</t>
@@ -1101,7 +1092,6 @@
           <t>Under $40 interior, under $150 coating</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
       <c r="D14" s="5" t="inlineStr">
         <is>
           <t>Cut ads that cost more after $50 spend.</t>
@@ -1119,7 +1109,6 @@
           <t>10 (Oct 2, Nov 3, Dec 5)</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
       <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Pitch a coating after every detail.</t>
@@ -1137,7 +1126,6 @@
           <t>10 by Dec 31 (launch Nov 1)</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
       <c r="D16" s="5" t="inlineStr">
         <is>
           <t>Offer to every happy customer.</t>
@@ -1155,7 +1143,6 @@
           <t>1 signed</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
       <c r="D17" s="5" t="inlineStr">
         <is>
           <t>Pitch 1 a week, push dealerships in December.</t>
@@ -1173,7 +1160,6 @@
           <t>Every customer, every 60 days</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
       <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Reactivation automation in GoHighLevel.</t>
@@ -1191,7 +1177,6 @@
           <t>10 referred jobs</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
       <c r="D19" s="5" t="inlineStr">
         <is>
           <t>$25 off for both people.</t>
@@ -1209,7 +1194,6 @@
           <t>50%+ every month</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
       <c r="D20" s="5" t="inlineStr">
         <is>
           <t>After tech pay, Rapid Reach, ads and supplies.</t>
@@ -1278,6 +1262,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -1323,7 +1308,6 @@
           <t>Separate business bank account + tax savings account. Start splitting every invoice.</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -1333,10 +1317,9 @@
       </c>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t>Rylan's $145 settled (paid back or taken from pay).</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr"/>
+          <t>Former tech's $145 settlement finalized (paid back or taken from pay).</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -1349,7 +1332,6 @@
           <t>Coating prices and packages set. Coating landing page built.</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -1362,7 +1344,6 @@
           <t>All techs trained on coating prep and paint correction.</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1375,7 +1356,6 @@
           <t>(Scratched — Meta ads plan dropped. Keep closing leads from LSA for the rest of October.)</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
@@ -1388,7 +1368,6 @@
           <t>All GoHighLevel automations live (instant text, missed-call, reminders, reviews, follow-ups).</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
@@ -1401,7 +1380,6 @@
           <t>October closed at $10k–12k. 65 reviews.</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
@@ -1414,7 +1392,6 @@
           <t>Winter Interior Reset ($250) + Google Search ad + maintenance plan launch.</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1427,7 +1404,6 @@
           <t>Black Friday gift card sale. Text every past customer.</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1440,7 +1416,6 @@
           <t>November closed at $20k. 95 reviews.</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1453,7 +1428,6 @@
           <t>UGA students and parents before winter break. Pitch dealerships.</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1466,7 +1440,6 @@
           <t>Last gift card push.</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1479,7 +1452,6 @@
           <t>December closed at $25k. 125 reviews. Write the 2027 plan.</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Log 40 Google reviews; team is Austin and Mo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XeYkWCpV7g2ezgB3AXjkpD
</commit_message>
<xml_diff>
--- a/Coastline_Goals_Sep_Dec_2026.xlsx
+++ b/Coastline_Goals_Sep_Dec_2026.xlsx
@@ -705,7 +705,9 @@
       <c r="K7" s="5" t="n">
         <v>65</v>
       </c>
-      <c r="L7" s="9" t="inlineStr"/>
+      <c r="L7" s="9" t="n">
+        <v>40</v>
+      </c>
       <c r="M7" s="6" t="n">
         <v>5000</v>
       </c>
@@ -918,6 +920,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
@@ -953,7 +956,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t>29</t>
+          <t>40</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">

</xml_diff>